<commit_message>
modified: Checklist e Planejamento
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/Hobby Hub - Checklist Verificacao de Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/Hobby Hub - Checklist Verificacao de Projeto.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550A178B-036A-4C06-B9E9-D7447A66A200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724DE22C-18F9-4E40-B969-107946BC8C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="666" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="666" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicadores" sheetId="6" r:id="rId1"/>
@@ -710,7 +710,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="117">
   <si>
     <t>Ambiente</t>
   </si>
@@ -1462,6 +1462,7 @@
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1513,7 +1514,6 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1620,7 +1620,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2583,10 +2583,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2595,22 +2595,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.83333333333333337</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2919,7 +2919,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2928,7 +2928,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2943,13 +2943,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>0.16666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7309,10 +7309,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="18">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="40"/>
+      <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="18" t="s">
@@ -7335,9 +7335,9 @@
       <c r="A4" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="20" t="e">
+      <c r="B4" s="20">
         <f>'Ver-Elaboração1'!$F$2</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -7440,21 +7440,21 @@
       <c r="N2" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="25" t="e">
+      <c r="O2" s="25">
         <f>('Ver-Elaboração1'!$G$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="P2" s="25">
         <f>('Ver-Elaboração1'!$H$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="25">
         <f>('Ver-Elaboração1'!$I$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R2" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R2" s="25">
         <f>('Ver-Elaboração1'!$J$6/SUM('Ver-Elaboração1'!$G$6:'Ver-Elaboração1'!$J$6))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -7480,21 +7480,21 @@
       <c r="N3" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="25" t="e">
+      <c r="O3" s="25">
         <f>('Ver-Elaboração1'!$G$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P3" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="P3" s="25">
         <f>('Ver-Elaboração1'!$H$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q3" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="25">
         <f>('Ver-Elaboração1'!$I$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R3" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R3" s="25">
         <f>('Ver-Elaboração1'!$J$8/SUM('Ver-Elaboração1'!$G$8:'Ver-Elaboração1'!$J$8))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -7520,21 +7520,21 @@
       <c r="N4" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="25" t="e">
+      <c r="O4" s="25">
         <f>('Ver-Elaboração1'!$G$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P4" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="P4" s="25">
         <f>('Ver-Elaboração1'!$H$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q4" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="25">
         <f>('Ver-Elaboração1'!$I$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R4" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R4" s="25">
         <f>('Ver-Elaboração1'!$J$11/SUM('Ver-Elaboração1'!$G$11:'Ver-Elaboração1'!$J$11))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -7560,21 +7560,21 @@
       <c r="N5" t="s">
         <v>4</v>
       </c>
-      <c r="O5" s="25" t="e">
+      <c r="O5" s="25">
         <f>('Ver-Elaboração1'!$G$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="P5" s="25">
         <f>('Ver-Elaboração1'!$H$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="25">
         <f>('Ver-Elaboração1'!$I$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R5" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R5" s="25">
         <f>('Ver-Elaboração1'!$J$16/SUM('Ver-Elaboração1'!$G$16:'Ver-Elaboração1'!$J$16))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -7640,21 +7640,21 @@
       <c r="N7" t="s">
         <v>5</v>
       </c>
-      <c r="O7" s="25" t="e">
+      <c r="O7" s="25">
         <f>('Ver-Elaboração1'!$G$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P7" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="P7" s="25">
         <f>('Ver-Elaboração1'!$H$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q7" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="25">
         <f>('Ver-Elaboração1'!$I$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R7" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R7" s="25">
         <f>('Ver-Elaboração1'!$J$18/SUM('Ver-Elaboração1'!$G$18:'Ver-Elaboração1'!$J$18))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -7720,21 +7720,21 @@
       <c r="N9" t="s">
         <v>6</v>
       </c>
-      <c r="O9" s="25" t="e">
+      <c r="O9" s="25">
         <f>('Ver-Elaboração1'!$G$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P9" s="25" t="e">
+        <v>1</v>
+      </c>
+      <c r="P9" s="25">
         <f>('Ver-Elaboração1'!$H$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q9" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="25">
         <f>('Ver-Elaboração1'!$I$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R9" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R9" s="25">
         <f>('Ver-Elaboração1'!$J$23/SUM('Ver-Elaboração1'!$G$23:'Ver-Elaboração1'!$J$23))</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -7760,21 +7760,21 @@
       <c r="N10" t="s">
         <v>13</v>
       </c>
-      <c r="O10" s="25" t="e">
+      <c r="O10" s="25">
         <f>('Ver-Elaboração1'!$G$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P10" s="25" t="e">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="P10" s="25">
         <f>('Ver-Elaboração1'!$H$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q10" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="25">
         <f>('Ver-Elaboração1'!$I$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R10" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R10" s="25">
         <f>('Ver-Elaboração1'!$J$29/SUM('Ver-Elaboração1'!$G$29:'Ver-Elaboração1'!$J$29))</f>
-        <v>#DIV/0!</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -7800,21 +7800,21 @@
       <c r="N11" t="s">
         <v>56</v>
       </c>
-      <c r="O11" s="25" t="e">
+      <c r="O11" s="25">
         <f>('Ver-Elaboração1'!$G$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P11" s="25" t="e">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="P11" s="25">
         <f>('Ver-Elaboração1'!$H$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q11" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="25">
         <f>('Ver-Elaboração1'!$I$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R11" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R11" s="25">
         <f>('Ver-Elaboração1'!$J$36/SUM('Ver-Elaboração1'!$G$36:'Ver-Elaboração1'!$J$36))</f>
-        <v>#DIV/0!</v>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -7840,21 +7840,21 @@
       <c r="N12" t="s">
         <v>15</v>
       </c>
-      <c r="O12" s="25" t="e">
+      <c r="O12" s="25">
         <f>('Ver-Elaboração1'!$G$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P12" s="25" t="e">
+        <v>0.5</v>
+      </c>
+      <c r="P12" s="25">
         <f>('Ver-Elaboração1'!$H$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q12" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="25">
         <f>('Ver-Elaboração1'!$I$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R12" s="25" t="e">
+        <v>0</v>
+      </c>
+      <c r="R12" s="25">
         <f>('Ver-Elaboração1'!$J$40/SUM('Ver-Elaboração1'!$G$40:'Ver-Elaboração1'!$J$40))</f>
-        <v>#DIV/0!</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -8421,45 +8421,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="45">
+      <c r="B2" s="33"/>
+      <c r="C2" s="28">
         <v>46263</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="39"/>
+      <c r="E2" s="40"/>
       <c r="F2" s="21">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="32"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="36"/>
-      <c r="F3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="38"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -8482,7 +8482,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="14.4">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="34" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="9"/>
@@ -8510,7 +8510,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="34"/>
+      <c r="A6" s="35"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -8524,7 +8524,7 @@
       <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="9"/>
@@ -8552,7 +8552,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1">
-      <c r="A8" s="30"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="22">
         <v>2</v>
       </c>
@@ -8566,7 +8566,7 @@
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="30"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
@@ -8580,7 +8580,7 @@
       <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:10" ht="14.4">
-      <c r="A10" s="30"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="5">
         <v>4</v>
       </c>
@@ -8594,7 +8594,7 @@
       <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A11" s="30"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="5">
         <v>5</v>
       </c>
@@ -8608,7 +8608,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A12" s="30"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="5">
         <v>6</v>
       </c>
@@ -8622,7 +8622,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="30"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>3</v>
@@ -8648,7 +8648,7 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8">
-      <c r="A14" s="30"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="23">
         <v>7</v>
       </c>
@@ -8662,7 +8662,7 @@
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A15" s="30"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="5">
         <v>8</v>
       </c>
@@ -8676,7 +8676,7 @@
       <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A16" s="30"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>9</v>
       </c>
@@ -8690,7 +8690,7 @@
       <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A17" s="30"/>
+      <c r="A17" s="31"/>
       <c r="B17" s="23">
         <v>10</v>
       </c>
@@ -8704,7 +8704,7 @@
       <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:10" s="1" customFormat="1" ht="14.4">
-      <c r="A18" s="30"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
@@ -8718,7 +8718,7 @@
       <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:10" ht="14.4">
-      <c r="A19" s="30"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="9"/>
       <c r="C19" s="10" t="s">
         <v>97</v>
@@ -8744,7 +8744,7 @@
       </c>
     </row>
     <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="30"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="23">
         <v>12</v>
       </c>
@@ -8758,7 +8758,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="28.8">
-      <c r="A21" s="30"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -8772,7 +8772,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="30"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="9"/>
       <c r="C22" s="10" t="s">
         <v>4</v>
@@ -8798,7 +8798,7 @@
       </c>
     </row>
     <row r="23" spans="1:10" ht="28.8">
-      <c r="A23" s="30"/>
+      <c r="A23" s="31"/>
       <c r="B23" s="23">
         <v>14</v>
       </c>
@@ -8812,7 +8812,7 @@
       <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:10" ht="14.4">
-      <c r="A24" s="30"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
@@ -8826,7 +8826,7 @@
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" ht="14.4">
-      <c r="A25" s="30"/>
+      <c r="A25" s="31"/>
       <c r="B25" s="9"/>
       <c r="C25" s="10" t="s">
         <v>36</v>
@@ -8852,7 +8852,7 @@
       </c>
     </row>
     <row r="26" spans="1:10" ht="28.8">
-      <c r="A26" s="30"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="23">
         <v>16</v>
       </c>
@@ -8866,7 +8866,7 @@
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="30"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>17</v>
       </c>
@@ -8880,7 +8880,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="30"/>
+      <c r="A28" s="31"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>13</v>
@@ -8906,7 +8906,7 @@
       </c>
     </row>
     <row r="29" spans="1:10" ht="28.8">
-      <c r="A29" s="30"/>
+      <c r="A29" s="31"/>
       <c r="B29" s="23">
         <v>21</v>
       </c>
@@ -8920,7 +8920,7 @@
       <c r="F29" s="8"/>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="30"/>
+      <c r="A30" s="31"/>
       <c r="B30" s="5">
         <v>22</v>
       </c>
@@ -8934,7 +8934,7 @@
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:10" ht="14.4">
-      <c r="A31" s="30"/>
+      <c r="A31" s="31"/>
       <c r="B31" s="5">
         <v>23</v>
       </c>
@@ -8948,7 +8948,7 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="30"/>
+      <c r="A32" s="31"/>
       <c r="B32" s="5">
         <v>24</v>
       </c>
@@ -8962,7 +8962,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="30"/>
+      <c r="A33" s="31"/>
       <c r="B33" s="5">
         <v>25</v>
       </c>
@@ -8976,7 +8976,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="30"/>
+      <c r="A34" s="31"/>
       <c r="B34" s="5">
         <v>26</v>
       </c>
@@ -8989,7 +8989,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A35" s="30"/>
+      <c r="A35" s="31"/>
       <c r="B35" s="5">
         <v>27</v>
       </c>
@@ -9003,7 +9003,7 @@
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="14.4">
-      <c r="A36" s="30"/>
+      <c r="A36" s="31"/>
       <c r="B36" s="5">
         <v>28</v>
       </c>
@@ -9017,7 +9017,7 @@
       <c r="F36" s="8"/>
     </row>
     <row r="37" spans="1:10" ht="15" customHeight="1">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B37" s="9"/>
@@ -9045,7 +9045,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="29"/>
+      <c r="A38" s="30"/>
       <c r="B38" s="23">
         <v>30</v>
       </c>
@@ -9059,7 +9059,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="29"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="5">
         <v>31</v>
       </c>
@@ -9073,7 +9073,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="29"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
@@ -9087,7 +9087,7 @@
       <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="28.8">
-      <c r="A41" s="29"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -9138,41 +9138,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="32"/>
+      <c r="B2" s="33"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="21" t="e">
+      <c r="E2" s="40"/>
+      <c r="F2" s="21">
         <f>COUNTIF(D5:D41,"Sim")/(COUNTA(D5:D42)-COUNTIF(D5:D42,"NA"))</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="32"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -9195,7 +9195,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9207,14 +9207,16 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="30"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6">
@@ -9231,11 +9233,11 @@
       </c>
       <c r="J6">
         <f>COUNTIF(D6,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="30"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9245,19 +9247,21 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="30"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8">
         <f>COUNTIF(D8,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8">
         <f>COUNTIF(D8,"Parcialmente")</f>
@@ -9273,14 +9277,16 @@
       </c>
     </row>
     <row r="9" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A9" s="30"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="5">
         <v>3</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9"/>
@@ -9289,7 +9295,7 @@
       <c r="J9"/>
     </row>
     <row r="10" spans="1:10" ht="14.4">
-      <c r="A10" s="30"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="9"/>
       <c r="C10" s="10" t="s">
         <v>97</v>
@@ -9299,19 +9305,21 @@
       <c r="F10" s="12"/>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="30"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="23">
         <v>4</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
       <c r="G11">
         <f>COUNTIF(D11:D14,"Sim")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H11">
         <f>COUNTIF(D11:D14,"Parcialmente")</f>
@@ -9327,43 +9335,49 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="28.8">
-      <c r="A12" s="30"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="23">
         <v>5</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="30"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="5">
         <v>6</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:10" ht="28.8">
-      <c r="A14" s="30"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="5">
         <v>7</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:10" ht="14.4">
-      <c r="A15" s="30"/>
+      <c r="A15" s="31"/>
       <c r="B15" s="9"/>
       <c r="C15" s="10" t="s">
         <v>4</v>
@@ -9373,14 +9387,16 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="30"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>7</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
       <c r="G16">
@@ -9397,11 +9413,11 @@
       </c>
       <c r="J16">
         <f>COUNTIF(D16,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="34" t="s">
         <v>18</v>
       </c>
       <c r="B17" s="9"/>
@@ -9413,19 +9429,21 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="28.8">
-      <c r="A18" s="30"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E18" s="8"/>
       <c r="F18" s="8"/>
       <c r="G18">
         <f>COUNTIF(D18:D21,"Sim")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
         <f>COUNTIF(D18:D21,"Parcialmente")</f>
@@ -9441,43 +9459,49 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="28.8">
-      <c r="A19" s="30"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="23">
         <v>10</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E19" s="8"/>
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A20" s="30"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E20" s="8"/>
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="28.8">
-      <c r="A21" s="30"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="5">
         <v>12</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E21" s="8"/>
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="34" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="9"/>
@@ -9489,19 +9513,21 @@
       <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="28.8">
-      <c r="A23" s="30"/>
+      <c r="A23" s="31"/>
       <c r="B23" s="5">
         <v>17</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
       <c r="G23">
         <f>COUNTIF(D23:D27,"Sim")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H23">
         <f>COUNTIF(D23:D27,"Parcialmente")</f>
@@ -9517,55 +9543,63 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="28.8">
-      <c r="A24" s="30"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="5">
         <v>18</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" ht="28.8">
-      <c r="A25" s="30"/>
+      <c r="A25" s="31"/>
       <c r="B25" s="5">
         <v>19</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="3"/>
+      <c r="D25" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E25" s="8"/>
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:10" ht="14.4">
-      <c r="A26" s="30"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="5">
         <v>21</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D26" s="3"/>
+      <c r="D26" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E26" s="8"/>
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="30"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>22</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D27" s="3"/>
+      <c r="D27" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="41" t="s">
+      <c r="A28" s="42" t="s">
         <v>11</v>
       </c>
       <c r="B28" s="9"/>
@@ -9577,19 +9611,21 @@
       <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="14.4">
-      <c r="A29" s="41"/>
+      <c r="A29" s="42"/>
       <c r="B29" s="5">
         <v>23</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D29" s="3"/>
+      <c r="D29" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E29" s="8"/>
       <c r="F29" s="8"/>
       <c r="G29">
         <f>COUNTIF(D29:D34,"Sim")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H29">
         <f>COUNTIF(D29:D34,"Parcialmente")</f>
@@ -9601,71 +9637,81 @@
       </c>
       <c r="J29">
         <f>COUNTIF(D29:D34,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="41"/>
+      <c r="A30" s="42"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D30" s="3"/>
+      <c r="D30" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E30" s="8"/>
       <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:10" ht="28.8">
-      <c r="A31" s="41"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="5">
         <v>25</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D31" s="3"/>
+      <c r="D31" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E31" s="8"/>
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="41"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="5">
         <v>26</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D32" s="3"/>
+      <c r="D32" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E32" s="8"/>
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="41"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="5">
         <v>27</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D33" s="3"/>
+      <c r="D33" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="41"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="5">
         <v>28</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D34" s="3"/>
+      <c r="D34" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E34" s="8"/>
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -9677,19 +9723,21 @@
       <c r="F35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="28.8">
-      <c r="A36" s="29"/>
+      <c r="A36" s="30"/>
       <c r="B36" s="5">
         <v>29</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D36" s="3"/>
+      <c r="D36" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E36" s="8"/>
       <c r="F36" s="8"/>
       <c r="G36">
         <f>COUNTIF(D36:D38,"Sim")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H36">
         <f>COUNTIF(D36:D38,"Parcialmente")</f>
@@ -9701,35 +9749,39 @@
       </c>
       <c r="J36">
         <f>COUNTIF(D36:D38,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="14.4">
-      <c r="A37" s="29"/>
+      <c r="A37" s="30"/>
       <c r="B37" s="5">
         <v>30</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D37" s="3"/>
+      <c r="D37" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E37" s="8"/>
       <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="29"/>
+      <c r="A38" s="30"/>
       <c r="B38" s="5">
         <v>31</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D38" s="3"/>
+      <c r="D38" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="E38" s="8"/>
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="29"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="9"/>
       <c r="C39" s="10" t="s">
         <v>15</v>
@@ -9739,19 +9791,21 @@
       <c r="F39" s="12"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="29"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="5">
         <v>32</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D40" s="3"/>
+      <c r="D40" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="E40" s="8"/>
       <c r="F40" s="8"/>
       <c r="G40">
         <f>COUNTIF(D40:D41,"Sim")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H40">
         <f>COUNTIF(D40:D41,"Parcialmente")</f>
@@ -9763,18 +9817,20 @@
       </c>
       <c r="J40">
         <f>COUNTIF(D40:D41,"NA")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="29"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D41" s="3"/>
+      <c r="D41" s="3" t="s">
+        <v>115</v>
+      </c>
       <c r="E41" s="8"/>
       <c r="F41" s="8"/>
     </row>
@@ -9819,41 +9875,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="32"/>
+      <c r="B2" s="33"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="39"/>
+      <c r="E2" s="40"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D42,"Sim")/(COUNTA(D5:D41)-COUNTIF(D5:D41,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="32"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -9876,7 +9932,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -9888,7 +9944,7 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="30"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -9916,7 +9972,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="30"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -9926,7 +9982,7 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="30"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -9954,7 +10010,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="30"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>97</v>
@@ -9964,7 +10020,7 @@
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:10" ht="28.8">
-      <c r="A10" s="30"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -9992,7 +10048,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="30"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -10004,7 +10060,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="18.75" customHeight="1">
-      <c r="A12" s="30"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -10016,7 +10072,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="30"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -10026,7 +10082,7 @@
       <c r="F13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="14.4">
-      <c r="A14" s="30"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -10054,7 +10110,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="34" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -10066,7 +10122,7 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="30"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10094,7 +10150,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="14.4">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="34" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10106,7 +10162,7 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="14.4">
-      <c r="A18" s="30"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>11</v>
       </c>
@@ -10134,7 +10190,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="28.8">
-      <c r="A19" s="30"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="5">
         <v>13</v>
       </c>
@@ -10146,7 +10202,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="30"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="5">
         <v>14</v>
       </c>
@@ -10158,7 +10214,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="14.4">
-      <c r="A21" s="30"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="5">
         <v>15</v>
       </c>
@@ -10170,7 +10226,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="30"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="5">
         <v>16</v>
       </c>
@@ -10182,7 +10238,7 @@
       <c r="F22" s="8"/>
     </row>
     <row r="23" spans="1:10" ht="14.4">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="34" t="s">
         <v>20</v>
       </c>
       <c r="B23" s="9"/>
@@ -10194,7 +10250,7 @@
       <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:10" ht="28.8">
-      <c r="A24" s="30"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="23">
         <v>17</v>
       </c>
@@ -10222,7 +10278,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" ht="28.8">
-      <c r="A25" s="30"/>
+      <c r="A25" s="31"/>
       <c r="B25" s="5">
         <v>18</v>
       </c>
@@ -10234,7 +10290,7 @@
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:10" ht="14.4">
-      <c r="A26" s="30"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="5">
         <v>19</v>
       </c>
@@ -10246,7 +10302,7 @@
       <c r="F26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="14.4">
-      <c r="A27" s="30"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>21</v>
       </c>
@@ -10258,7 +10314,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="30"/>
+      <c r="A28" s="31"/>
       <c r="B28" s="5">
         <v>22</v>
       </c>
@@ -10270,7 +10326,7 @@
       <c r="F28" s="8"/>
     </row>
     <row r="29" spans="1:10" ht="14.4">
-      <c r="A29" s="41" t="s">
+      <c r="A29" s="42" t="s">
         <v>11</v>
       </c>
       <c r="B29" s="9"/>
@@ -10282,7 +10338,7 @@
       <c r="F29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="41"/>
+      <c r="A30" s="42"/>
       <c r="B30" s="5">
         <v>24</v>
       </c>
@@ -10310,7 +10366,7 @@
       </c>
     </row>
     <row r="31" spans="1:10" ht="28.8">
-      <c r="A31" s="41"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="5">
         <v>26</v>
       </c>
@@ -10322,7 +10378,7 @@
       <c r="F31" s="8"/>
     </row>
     <row r="32" spans="1:10" ht="14.4">
-      <c r="A32" s="41"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="5">
         <v>27</v>
       </c>
@@ -10334,7 +10390,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="41"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="5">
         <v>28</v>
       </c>
@@ -10346,7 +10402,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="41"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="5">
         <v>29</v>
       </c>
@@ -10358,7 +10414,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="15" customHeight="1">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B35" s="9"/>
@@ -10370,7 +10426,7 @@
       <c r="F35" s="12"/>
     </row>
     <row r="36" spans="1:10" ht="28.8">
-      <c r="A36" s="29"/>
+      <c r="A36" s="30"/>
       <c r="B36" s="5">
         <v>30</v>
       </c>
@@ -10398,7 +10454,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" ht="14.4">
-      <c r="A37" s="29"/>
+      <c r="A37" s="30"/>
       <c r="B37" s="5">
         <v>31</v>
       </c>
@@ -10410,7 +10466,7 @@
       <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:10" ht="28.8">
-      <c r="A38" s="29"/>
+      <c r="A38" s="30"/>
       <c r="B38" s="5">
         <v>32</v>
       </c>
@@ -10422,7 +10478,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="14.4">
-      <c r="A39" s="29"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="5"/>
       <c r="C39" s="8" t="s">
         <v>105</v>
@@ -10432,7 +10488,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="29"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="9"/>
       <c r="C40" s="10" t="s">
         <v>15</v>
@@ -10442,7 +10498,7 @@
       <c r="F40" s="12"/>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="29"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="5">
         <v>33</v>
       </c>
@@ -10470,7 +10526,7 @@
       </c>
     </row>
     <row r="42" spans="1:10" ht="14.4">
-      <c r="A42" s="29"/>
+      <c r="A42" s="30"/>
       <c r="B42" s="5">
         <v>34</v>
       </c>
@@ -10511,17 +10567,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:F3"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A17:A22"/>
     <mergeCell ref="A29:A34"/>
     <mergeCell ref="A35:A42"/>
     <mergeCell ref="A23:A28"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:F3"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23 D15 D17 D40 D35 D29" xr:uid="{00000000-0002-0000-0300-000000000000}">
@@ -10551,41 +10607,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="19.5" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="32"/>
+      <c r="B2" s="33"/>
       <c r="C2" s="16"/>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="39"/>
+      <c r="E2" s="40"/>
       <c r="F2" s="21" t="e">
         <f>COUNTIF(D5:D43,"Sim")/(COUNTA(D5:D43)-COUNTIF(D5:D43,"NA"))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="32"/>
+      <c r="B3" s="33"/>
       <c r="C3" s="13"/>
-      <c r="D3" s="42" t="s">
+      <c r="D3" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="43"/>
-      <c r="F3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
     </row>
     <row r="4" spans="1:10" ht="14.4">
       <c r="A4" s="6" t="s">
@@ -10608,7 +10664,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="34" t="s">
         <v>17</v>
       </c>
       <c r="B5" s="9"/>
@@ -10620,7 +10676,7 @@
       <c r="F5" s="12"/>
     </row>
     <row r="6" spans="1:10" ht="14.4">
-      <c r="A6" s="30"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="5">
         <v>1</v>
       </c>
@@ -10648,7 +10704,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="14.4">
-      <c r="A7" s="30"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="9"/>
       <c r="C7" s="10" t="s">
         <v>3</v>
@@ -10658,7 +10714,7 @@
       <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A8" s="30"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="5">
         <v>2</v>
       </c>
@@ -10686,7 +10742,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="14.4">
-      <c r="A9" s="30"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10" t="s">
         <v>14</v>
@@ -10696,7 +10752,7 @@
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:10" ht="28.8">
-      <c r="A10" s="30"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="5">
         <v>3</v>
       </c>
@@ -10724,7 +10780,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="28.8">
-      <c r="A11" s="30"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="5">
         <v>4</v>
       </c>
@@ -10736,7 +10792,7 @@
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:10" ht="29.25" customHeight="1">
-      <c r="A12" s="30"/>
+      <c r="A12" s="31"/>
       <c r="B12" s="5">
         <v>5</v>
       </c>
@@ -10748,7 +10804,7 @@
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:10" ht="14.4">
-      <c r="A13" s="30"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="9"/>
       <c r="C13" s="10" t="s">
         <v>4</v>
@@ -10758,7 +10814,7 @@
       <c r="F13" s="12"/>
     </row>
     <row r="14" spans="1:10" ht="14.4">
-      <c r="A14" s="30"/>
+      <c r="A14" s="31"/>
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -10786,7 +10842,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" ht="15" customHeight="1">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="34" t="s">
         <v>18</v>
       </c>
       <c r="B15" s="9"/>
@@ -10798,7 +10854,7 @@
       <c r="F15" s="12"/>
     </row>
     <row r="16" spans="1:10" ht="14.4">
-      <c r="A16" s="30"/>
+      <c r="A16" s="31"/>
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -10826,7 +10882,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="34" t="s">
         <v>19</v>
       </c>
       <c r="B17" s="9"/>
@@ -10838,7 +10894,7 @@
       <c r="F17" s="12"/>
     </row>
     <row r="18" spans="1:10" ht="14.4">
-      <c r="A18" s="30"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="5">
         <v>9</v>
       </c>
@@ -10866,7 +10922,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" ht="14.4">
-      <c r="A19" s="30"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="5">
         <v>10</v>
       </c>
@@ -10878,7 +10934,7 @@
       <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:10" ht="28.8">
-      <c r="A20" s="30"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="5">
         <v>11</v>
       </c>
@@ -10890,7 +10946,7 @@
       <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:10" ht="14.4">
-      <c r="A21" s="34"/>
+      <c r="A21" s="35"/>
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -10902,7 +10958,7 @@
       <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:10" ht="14.4">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="34" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="9"/>
@@ -10914,7 +10970,7 @@
       <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:10" ht="14.4">
-      <c r="A23" s="30"/>
+      <c r="A23" s="31"/>
       <c r="B23" s="5">
         <v>14</v>
       </c>
@@ -10942,7 +10998,7 @@
       </c>
     </row>
     <row r="24" spans="1:10" ht="14.4">
-      <c r="A24" s="30"/>
+      <c r="A24" s="31"/>
       <c r="B24" s="5">
         <v>15</v>
       </c>
@@ -10954,7 +11010,7 @@
       <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:10" s="1" customFormat="1" ht="15" customHeight="1">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="34" t="s">
         <v>21</v>
       </c>
       <c r="B25" s="9"/>
@@ -10966,7 +11022,7 @@
       <c r="F25" s="12"/>
     </row>
     <row r="26" spans="1:10" s="1" customFormat="1" ht="28.8">
-      <c r="A26" s="30"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="23">
         <v>24</v>
       </c>
@@ -10994,7 +11050,7 @@
       </c>
     </row>
     <row r="27" spans="1:10" s="1" customFormat="1" ht="43.2">
-      <c r="A27" s="30"/>
+      <c r="A27" s="31"/>
       <c r="B27" s="5">
         <v>25</v>
       </c>
@@ -11006,7 +11062,7 @@
       <c r="F27" s="8"/>
     </row>
     <row r="28" spans="1:10" ht="14.4">
-      <c r="A28" s="30"/>
+      <c r="A28" s="31"/>
       <c r="B28" s="9"/>
       <c r="C28" s="10" t="s">
         <v>10</v>
@@ -11016,7 +11072,7 @@
       <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:10" ht="28.8">
-      <c r="A29" s="30"/>
+      <c r="A29" s="31"/>
       <c r="B29" s="23">
         <v>26</v>
       </c>
@@ -11044,7 +11100,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" ht="14.4">
-      <c r="A30" s="41" t="s">
+      <c r="A30" s="42" t="s">
         <v>11</v>
       </c>
       <c r="B30" s="9"/>
@@ -11056,7 +11112,7 @@
       <c r="F30" s="12"/>
     </row>
     <row r="31" spans="1:10" ht="14.4">
-      <c r="A31" s="41"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="5">
         <v>19</v>
       </c>
@@ -11084,7 +11140,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" ht="28.8">
-      <c r="A32" s="41"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="5">
         <v>20</v>
       </c>
@@ -11096,7 +11152,7 @@
       <c r="F32" s="8"/>
     </row>
     <row r="33" spans="1:10" ht="14.4">
-      <c r="A33" s="41"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="5">
         <v>21</v>
       </c>
@@ -11108,7 +11164,7 @@
       <c r="F33" s="8"/>
     </row>
     <row r="34" spans="1:10" ht="14.4">
-      <c r="A34" s="41"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="5">
         <v>24</v>
       </c>
@@ -11120,7 +11176,7 @@
       <c r="F34" s="8"/>
     </row>
     <row r="35" spans="1:10" ht="14.4">
-      <c r="A35" s="41"/>
+      <c r="A35" s="42"/>
       <c r="B35" s="5">
         <v>25</v>
       </c>
@@ -11132,7 +11188,7 @@
       <c r="F35" s="8"/>
     </row>
     <row r="36" spans="1:10" ht="15" customHeight="1">
-      <c r="A36" s="28" t="s">
+      <c r="A36" s="29" t="s">
         <v>30</v>
       </c>
       <c r="B36" s="9"/>
@@ -11144,7 +11200,7 @@
       <c r="F36" s="12"/>
     </row>
     <row r="37" spans="1:10" ht="28.8">
-      <c r="A37" s="29"/>
+      <c r="A37" s="30"/>
       <c r="B37" s="5">
         <v>26</v>
       </c>
@@ -11172,7 +11228,7 @@
       </c>
     </row>
     <row r="38" spans="1:10" ht="14.4">
-      <c r="A38" s="29"/>
+      <c r="A38" s="30"/>
       <c r="B38" s="5">
         <v>27</v>
       </c>
@@ -11184,7 +11240,7 @@
       <c r="F38" s="8"/>
     </row>
     <row r="39" spans="1:10" ht="28.8">
-      <c r="A39" s="29"/>
+      <c r="A39" s="30"/>
       <c r="B39" s="5">
         <v>28</v>
       </c>
@@ -11196,7 +11252,7 @@
       <c r="F39" s="8"/>
     </row>
     <row r="40" spans="1:10" ht="14.4">
-      <c r="A40" s="29"/>
+      <c r="A40" s="30"/>
       <c r="B40" s="5"/>
       <c r="C40" s="8" t="s">
         <v>105</v>
@@ -11206,7 +11262,7 @@
       <c r="F40" s="8"/>
     </row>
     <row r="41" spans="1:10" ht="14.4">
-      <c r="A41" s="29"/>
+      <c r="A41" s="30"/>
       <c r="B41" s="9"/>
       <c r="C41" s="10" t="s">
         <v>15</v>
@@ -11216,7 +11272,7 @@
       <c r="F41" s="12"/>
     </row>
     <row r="42" spans="1:10" ht="14.4">
-      <c r="A42" s="29"/>
+      <c r="A42" s="30"/>
       <c r="B42" s="5">
         <v>29</v>
       </c>
@@ -11244,7 +11300,7 @@
       </c>
     </row>
     <row r="43" spans="1:10" ht="14.4">
-      <c r="A43" s="29"/>
+      <c r="A43" s="30"/>
       <c r="B43" s="5">
         <v>30</v>
       </c>
@@ -11285,11 +11341,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A22:A24"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A43"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A25:A29"/>
     <mergeCell ref="A5:A14"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="A1:F1"/>
@@ -11297,6 +11348,11 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="D3:F3"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A43"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A25:A29"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D25 D17 D15 D22 D41 D36 D30 D28" xr:uid="{00000000-0002-0000-0400-000000000000}">

</xml_diff>